<commit_message>
Updated summary table of samples over chronic Cu tox threshold for Daph
</commit_message>
<xml_diff>
--- a/Copper/6. Statistical data analysis/Plots of Cu Toxicity/Relative_prop_on_above_tox_threshold.xlsx
+++ b/Copper/6. Statistical data analysis/Plots of Cu Toxicity/Relative_prop_on_above_tox_threshold.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ornl-my.sharepoint.com/personal/q4q_ornl_gov/Documents/Research/Bioavailability Project/Trace-element-bioavailability-spatial-assessment/Copper/6. Statistical data analysis/Plots of Cu Toxicity/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://irtacat-my.sharepoint.com/personal/cecilia_albert_irta_cat/Documents/Escriptori/Trace-element-bioavailability-spatial-assessment/Copper/6. Statistical data analysis/Plots of Cu Toxicity/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_BFD6FCEA77690FC81C4DEEB04816AF38B8F6B0CC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CAF0C1D3-42D5-4147-858C-035256693836}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_2FD4E62A5DA391F014AE1DA1C1EC019CE897B126" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFF4DCC0-4E3B-4591-842D-5D0CDCC6F068}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Chronic tox daphnia" sheetId="1" r:id="rId1"/>
@@ -20,14 +20,14 @@
     <sheet name="Acute tox minnow" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Samples chronic tox daph'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Samples chronic tox daph'!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="49">
   <si>
     <t>prop_chronic_tox_daph</t>
   </si>
@@ -53,6 +53,15 @@
     <t>Sample_ID</t>
   </si>
   <si>
+    <t>Regime</t>
+  </si>
+  <si>
+    <t>Flow_state</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
     <t>Typology</t>
   </si>
   <si>
@@ -87,6 +96,12 @@
   </si>
   <si>
     <t>Perennial</t>
+  </si>
+  <si>
+    <t>Flowing</t>
+  </si>
+  <si>
+    <t>Tributaries</t>
   </si>
   <si>
     <t>BCK0.9</t>
@@ -194,8 +209,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -545,10 +561,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26.36328125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -582,431 +614,548 @@
       <c r="K1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M1" t="s">
+        <v>18</v>
+      </c>
+      <c r="N1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
         <v>22</v>
       </c>
-      <c r="D2">
-        <v>2.2121876044039599</v>
-      </c>
-      <c r="E2">
-        <v>5.0549958615291404</v>
-      </c>
-      <c r="F2">
-        <v>7.93</v>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
       </c>
       <c r="G2">
-        <v>-6.7226089842574597</v>
+        <v>2.4983105537896</v>
       </c>
       <c r="H2">
-        <v>1.74772603274185</v>
+        <v>5.4585169850488304</v>
       </c>
       <c r="I2">
-        <v>-1.28384254170954</v>
+        <v>7.68</v>
       </c>
       <c r="J2">
-        <v>7.7248579851976501E-2</v>
+        <v>-6.7015094024105002</v>
       </c>
       <c r="K2">
-        <v>2.29815625559876</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+        <v>2.4666772802949</v>
+      </c>
+      <c r="L2">
+        <v>0.63471401941151895</v>
+      </c>
+      <c r="M2">
+        <v>-0.58206389603518804</v>
+      </c>
+      <c r="N2">
+        <v>2.3458133559801402</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3">
-        <v>2.4983105537896</v>
-      </c>
-      <c r="E3">
-        <v>5.4585169850488304</v>
-      </c>
-      <c r="F3">
-        <v>7.68</v>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" t="s">
+        <v>27</v>
       </c>
       <c r="G3">
-        <v>-6.7015094024105002</v>
+        <v>2.3117538610557502</v>
       </c>
       <c r="H3">
-        <v>2.4666772802949</v>
+        <v>5.1266508206674803</v>
       </c>
       <c r="I3">
-        <v>0.63471401941151895</v>
+        <v>7.55</v>
       </c>
       <c r="J3">
-        <v>-0.58206389603518804</v>
+        <v>-6.4066877554731096</v>
       </c>
       <c r="K3">
-        <v>2.3458133559801402</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+        <v>1.9979096848665601</v>
+      </c>
+      <c r="L3">
+        <v>-0.94315630751041502</v>
+      </c>
+      <c r="M3">
+        <v>-0.924906383496513</v>
+      </c>
+      <c r="N3">
+        <v>3.0117196722573301</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
         <v>22</v>
       </c>
-      <c r="D4">
-        <v>2.2329961103921501</v>
-      </c>
-      <c r="E4">
-        <v>5.0549958615291404</v>
-      </c>
-      <c r="F4">
-        <v>7.72</v>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
       </c>
       <c r="G4">
-        <v>-6.5061397425595597</v>
+        <v>2.1643528557844398</v>
       </c>
       <c r="H4">
-        <v>1.8000123011871001</v>
+        <v>5.10002573010786</v>
       </c>
       <c r="I4">
-        <v>-1.28384254170954</v>
+        <v>7.77</v>
       </c>
       <c r="J4">
-        <v>-0.476573899893242</v>
+        <v>-6.7402603647577299</v>
       </c>
       <c r="K4">
-        <v>2.78708994423316</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+        <v>1.62752996923058</v>
+      </c>
+      <c r="L4">
+        <v>-1.06974631533465</v>
+      </c>
+      <c r="M4">
+        <v>-0.34471140471580902</v>
+      </c>
+      <c r="N4">
+        <v>2.2582875217786902</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
         <v>22</v>
       </c>
-      <c r="D5">
-        <v>2.3117538610557502</v>
-      </c>
-      <c r="E5">
-        <v>5.1266508206674803</v>
-      </c>
-      <c r="F5">
-        <v>7.55</v>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" t="s">
+        <v>27</v>
       </c>
       <c r="G5">
-        <v>-6.4066877554731096</v>
+        <v>2.5998830720736898</v>
       </c>
       <c r="H5">
-        <v>1.9979096848665601</v>
+        <v>5.4301879703434901</v>
       </c>
       <c r="I5">
-        <v>-0.94315630751041502</v>
+        <v>7.48</v>
       </c>
       <c r="J5">
-        <v>-0.924906383496513</v>
+        <v>-6.2707860203011601</v>
       </c>
       <c r="K5">
-        <v>3.0117196722573301</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+        <v>2.7219021369316998</v>
+      </c>
+      <c r="L5">
+        <v>0.500022639295024</v>
+      </c>
+      <c r="M5">
+        <v>-1.10951387674492</v>
+      </c>
+      <c r="N5">
+        <v>3.3186775391036898</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
       </c>
-      <c r="D6">
-        <v>2.1643528557844398</v>
-      </c>
-      <c r="E6">
-        <v>5.10002573010786</v>
-      </c>
-      <c r="F6">
-        <v>7.77</v>
+      <c r="D6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" t="s">
+        <v>27</v>
       </c>
       <c r="G6">
-        <v>-6.7402603647577299</v>
+        <v>2.3802112417116099</v>
       </c>
       <c r="H6">
-        <v>1.62752996923058</v>
+        <v>5.2776779626062504</v>
       </c>
       <c r="I6">
-        <v>-1.06974631533465</v>
+        <v>7.59</v>
       </c>
       <c r="J6">
-        <v>-0.34471140471580902</v>
+        <v>-6.4633051839245104</v>
       </c>
       <c r="K6">
-        <v>2.2582875217786902</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+        <v>2.1699249647748</v>
+      </c>
+      <c r="L6">
+        <v>-0.22509200508523999</v>
+      </c>
+      <c r="M6">
+        <v>-0.81941638735456701</v>
+      </c>
+      <c r="N6">
+        <v>2.88383929573543</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s">
         <v>22</v>
       </c>
-      <c r="D7">
-        <v>2.5998830720736898</v>
-      </c>
-      <c r="E7">
-        <v>5.4301879703434901</v>
-      </c>
-      <c r="F7">
-        <v>7.48</v>
+      <c r="D7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" t="s">
+        <v>27</v>
       </c>
       <c r="G7">
-        <v>-6.2707860203011601</v>
+        <v>2.18184358794477</v>
       </c>
       <c r="H7">
-        <v>2.7219021369316998</v>
+        <v>5.3291333572142898</v>
       </c>
       <c r="I7">
-        <v>0.500022639295024</v>
+        <v>7.54</v>
       </c>
       <c r="J7">
-        <v>-1.10951387674492</v>
+        <v>-6.7008512275368401</v>
       </c>
       <c r="K7">
-        <v>3.3186775391036898</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+        <v>1.6714795501163</v>
+      </c>
+      <c r="L7">
+        <v>1.9554629691266399E-2</v>
+      </c>
+      <c r="M7">
+        <v>-0.95127888253199899</v>
+      </c>
+      <c r="N7">
+        <v>2.34729995918631</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="1">
+        <v>2.2121876044039599</v>
+      </c>
+      <c r="H8" s="1">
+        <v>5.0549958615291404</v>
+      </c>
+      <c r="I8" s="1">
+        <v>7.93</v>
+      </c>
+      <c r="J8" s="1">
+        <v>-6.7226089842574597</v>
+      </c>
+      <c r="K8" s="1">
+        <v>1.74772603274185</v>
+      </c>
+      <c r="L8" s="1">
+        <v>-1.28384254170954</v>
+      </c>
+      <c r="M8" s="1">
+        <v>7.7248579851976501E-2</v>
+      </c>
+      <c r="N8" s="1">
+        <v>2.29815625559876</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="1">
+        <v>2.2329961103921501</v>
+      </c>
+      <c r="H9" s="1">
+        <v>5.0549958615291404</v>
+      </c>
+      <c r="I9" s="1">
+        <v>7.72</v>
+      </c>
+      <c r="J9" s="1">
+        <v>-6.5061397425595597</v>
+      </c>
+      <c r="K9" s="1">
+        <v>1.8000123011871001</v>
+      </c>
+      <c r="L9" s="1">
+        <v>-1.28384254170954</v>
+      </c>
+      <c r="M9" s="1">
+        <v>-0.476573899893242</v>
+      </c>
+      <c r="N9" s="1">
+        <v>2.78708994423316</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10">
+        <v>1.0899051114394001</v>
+      </c>
+      <c r="H10">
+        <v>4.6073477767684103</v>
+      </c>
+      <c r="I10">
+        <v>6.87</v>
+      </c>
+      <c r="J10">
+        <v>-6.5900703052143204</v>
+      </c>
+      <c r="K10">
+        <v>0.51555903550316795</v>
+      </c>
+      <c r="L10">
+        <v>-2.3633671160395999</v>
+      </c>
+      <c r="M10">
+        <v>-1.96531168366773</v>
+      </c>
+      <c r="N10">
+        <v>2.72863582433797</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11">
+        <v>2.4593924877592301</v>
+      </c>
+      <c r="H11">
+        <v>5.1068365873667902</v>
+      </c>
+      <c r="I11">
+        <v>7.66</v>
+      </c>
+      <c r="J11">
+        <v>-6.2075103291393701</v>
+      </c>
+      <c r="K11">
+        <v>3.1198969598063102</v>
+      </c>
+      <c r="L11">
+        <v>-0.44868884580141999</v>
+      </c>
+      <c r="M11">
+        <v>0.262607609636825</v>
+      </c>
+      <c r="N11">
+        <v>3.45129929491875</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
         <v>38</v>
       </c>
-      <c r="B8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8">
-        <v>2.3802112417116099</v>
-      </c>
-      <c r="E8">
-        <v>5.2776779626062504</v>
-      </c>
-      <c r="F8">
-        <v>7.59</v>
-      </c>
-      <c r="G8">
-        <v>-6.4633051839245104</v>
-      </c>
-      <c r="H8">
-        <v>2.1699249647748</v>
-      </c>
-      <c r="I8">
-        <v>-0.22509200508523999</v>
-      </c>
-      <c r="J8">
-        <v>-0.81941638735456701</v>
-      </c>
-      <c r="K8">
-        <v>2.88383929573543</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9">
-        <v>2.18184358794477</v>
-      </c>
-      <c r="E9">
-        <v>5.3291333572142898</v>
-      </c>
-      <c r="F9">
-        <v>7.54</v>
-      </c>
-      <c r="G9">
-        <v>-6.7008512275368401</v>
-      </c>
-      <c r="H9">
-        <v>1.6714795501163</v>
-      </c>
-      <c r="I9">
-        <v>1.9554629691266399E-2</v>
-      </c>
-      <c r="J9">
-        <v>-0.95127888253199899</v>
-      </c>
-      <c r="K9">
-        <v>2.34729995918631</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10">
-        <v>1.0899051114394001</v>
-      </c>
-      <c r="E10">
-        <v>4.6073477767684103</v>
-      </c>
-      <c r="F10">
-        <v>6.87</v>
-      </c>
-      <c r="G10">
-        <v>-6.5900703052143204</v>
-      </c>
-      <c r="H10">
-        <v>0.51555903550316795</v>
-      </c>
-      <c r="I10">
-        <v>-2.3633671160395999</v>
-      </c>
-      <c r="J10">
-        <v>-1.96531168366773</v>
-      </c>
-      <c r="K10">
-        <v>2.72863582433797</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11">
-        <v>2.4593924877592301</v>
-      </c>
-      <c r="E11">
-        <v>5.1068365873667902</v>
-      </c>
-      <c r="F11">
-        <v>7.66</v>
-      </c>
-      <c r="G11">
-        <v>-6.2075103291393701</v>
-      </c>
-      <c r="H11">
-        <v>3.1198969598063102</v>
-      </c>
-      <c r="I11">
-        <v>-0.44868884580141999</v>
-      </c>
-      <c r="J11">
-        <v>0.262607609636825</v>
-      </c>
-      <c r="K11">
-        <v>3.45129929491875</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" t="s">
-        <v>33</v>
-      </c>
       <c r="C12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12">
+        <v>22</v>
+      </c>
+      <c r="D12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12">
         <v>2.1367205671564098</v>
       </c>
-      <c r="E12">
+      <c r="H12">
         <v>5.3880301164599702</v>
       </c>
-      <c r="F12">
+      <c r="I12">
         <v>7.47</v>
       </c>
-      <c r="G12">
+      <c r="J12">
         <v>-6.7222649230832703</v>
       </c>
-      <c r="H12">
+      <c r="K12">
         <v>2.5062755898949698</v>
       </c>
-      <c r="I12">
+      <c r="L12">
         <v>0.62920344820474805</v>
       </c>
-      <c r="J12">
+      <c r="M12">
         <v>-0.27322108115794203</v>
       </c>
-      <c r="K12">
+      <c r="N12">
         <v>2.4789175387989699</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>19</v>
-      </c>
-      <c r="D13">
+        <v>22</v>
+      </c>
+      <c r="D13" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" t="s">
+        <v>22</v>
+      </c>
+      <c r="G13">
         <v>2.0530784434834199</v>
       </c>
-      <c r="E13">
+      <c r="H13">
         <v>5.3496077377480704</v>
       </c>
-      <c r="F13">
+      <c r="I13">
         <v>7.39</v>
       </c>
-      <c r="G13">
+      <c r="J13">
         <v>-6.7220623177931396</v>
       </c>
-      <c r="H13">
+      <c r="K13">
         <v>2.3472143539044699</v>
       </c>
-      <c r="I13">
+      <c r="L13">
         <v>0.48191988138689501</v>
       </c>
-      <c r="J13">
+      <c r="M13">
         <v>-0.49883316149258</v>
       </c>
-      <c r="K13">
+      <c r="N13">
         <v>2.4793002642571502</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1" xr:uid="{00000000-0001-0000-0100-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K13">
-      <sortCondition ref="C1"/>
+  <autoFilter ref="A1:N1" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N13">
+      <sortCondition ref="F1"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1021,7 +1170,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1060,7 +1209,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1099,7 +1248,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>

</xml_diff>